<commit_message>
SLR dia 1: distancia recorrida; Discusion sin el nivel de azar
- Distancia por minuto del muestreo (ANOVA de dos vias por configuracion + Tukey), panel B de fig:slr-dia1
- Discusion: se quitan las afirmaciones contra el azar y se agrega el efecto de cohorte en la distancia
- IHC: Excel con el DCX de Prism ya con Tukey (coincide con el texto)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Resultados inmucitoquimica/IHC_para_Prism_Grouped.xlsx
+++ b/Resultados inmucitoquimica/IHC_para_Prism_Grouped.xlsx
@@ -8,21 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Thiago\tesis-pfc\Resultados inmucitoquimica\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48A71DBA-495B-4335-B3E8-5662C1C2C112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E08B35B-5A9D-4DFD-B8FB-DC4D66D4D571}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PCNA" sheetId="1" r:id="rId1"/>
     <sheet name="DCX" sheetId="2" r:id="rId2"/>
     <sheet name="PCNA+DCX" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="179">
   <si>
     <t>PCNA: copiar el bloque amarillo (B3:AO4) y pegarlo en Prism en la tabla Grouped, celda de la fila 'Juvenil', columna A (Control), primera subcolumna.</t>
   </si>
@@ -327,9 +327,6 @@
     <t>Alpha</t>
   </si>
   <si>
-    <t>Šídák's multiple comparisons test</t>
-  </si>
-  <si>
     <t>Mean diff.</t>
   </si>
   <si>
@@ -348,36 +345,21 @@
     <t>  Juvenil:Control  vs. Juvenil:Sacarosa</t>
   </si>
   <si>
-    <t>-1935 to 2985</t>
-  </si>
-  <si>
     <t>  Juvenil:Control  vs. Adulto:Control </t>
   </si>
   <si>
-    <t>-1410 to 3510</t>
-  </si>
-  <si>
     <t>  Juvenil:Control  vs. Adulto:Sacarosa</t>
   </si>
   <si>
-    <t>-3195 to 1725</t>
-  </si>
-  <si>
     <t>  Juvenil:Sacarosa vs. Adulto:Control </t>
   </si>
   <si>
     <t>  Juvenil:Sacarosa vs. Adulto:Sacarosa</t>
   </si>
   <si>
-    <t>-3720 to 1200</t>
-  </si>
-  <si>
     <t>  Adulto:Control  vs. Adulto:Sacarosa</t>
   </si>
   <si>
-    <t>-4245 to 674.8</t>
-  </si>
-  <si>
     <t>Test details</t>
   </si>
   <si>
@@ -396,9 +378,6 @@
     <t>N2</t>
   </si>
   <si>
-    <t>t</t>
-  </si>
-  <si>
     <t>Compact letter display</t>
   </si>
   <si>
@@ -565,6 +544,21 @@
   </si>
   <si>
     <t>  Juvenil:Sucarosa</t>
+  </si>
+  <si>
+    <t>-1867 to 2917</t>
+  </si>
+  <si>
+    <t>-1342 to 3442</t>
+  </si>
+  <si>
+    <t>-3127 to 1657</t>
+  </si>
+  <si>
+    <t>-3652 to 1132</t>
+  </si>
+  <si>
+    <t>-4177 to 607.0</t>
   </si>
 </sst>
 </file>
@@ -1502,29 +1496,29 @@
         <v>3.1800000000000002E-2</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="G16" s="3"/>
       <c r="I16" s="5" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="J16" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="K16" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="K16" s="3" t="s">
+      <c r="L16" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="L16" s="3" t="s">
+      <c r="M16" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="M16" s="3" t="s">
+      <c r="N16" s="3" t="s">
         <v>105</v>
-      </c>
-      <c r="N16" s="3" t="s">
-        <v>106</v>
       </c>
       <c r="O16" s="3"/>
       <c r="P16" s="3"/>
@@ -1541,10 +1535,10 @@
         <v>2.9999999999999997E-4</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="G17" s="3"/>
       <c r="I17" s="5"/>
@@ -1565,13 +1559,13 @@
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
       <c r="I18" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="J18" s="3">
         <v>599.29999999999995</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="L18" s="3" t="s">
         <v>59</v>
@@ -1606,13 +1600,13 @@
         <v>54</v>
       </c>
       <c r="I19" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="J19" s="3">
         <v>314.3</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="L19" s="3" t="s">
         <v>59</v>
@@ -1641,25 +1635,25 @@
         <v>92820</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="J20" s="3">
         <v>1050</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="N20" s="3">
         <v>2.9999999999999997E-4</v>
@@ -1682,19 +1676,19 @@
         <v>2924978</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="J21" s="3">
         <v>-285</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="L21" s="3" t="s">
         <v>59</v>
@@ -1723,19 +1717,19 @@
         <v>8907788</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="I22" s="5" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="J22" s="3">
         <v>450.6</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="L22" s="3" t="s">
         <v>59</v>
@@ -1766,19 +1760,19 @@
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
       <c r="I23" s="5" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="J23" s="3">
         <v>735.5</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="N23" s="3">
         <v>2.01E-2</v>
@@ -1837,28 +1831,28 @@
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
       <c r="I26" s="5" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="L26" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M26" s="3" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="N26" s="3" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="O26" s="3" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="P26" s="3" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="Q26" s="3" t="s">
         <v>64</v>
@@ -1897,7 +1891,7 @@
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
       <c r="I28" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="J28" s="3">
         <v>2310</v>
@@ -1936,7 +1930,7 @@
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
       <c r="I29" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="J29" s="3">
         <v>2310</v>
@@ -1975,7 +1969,7 @@
       <c r="F30" s="3"/>
       <c r="G30" s="3"/>
       <c r="I30" s="5" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="J30" s="3">
         <v>2310</v>
@@ -2007,14 +2001,14 @@
         <v>80</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="D31" s="3"/>
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
       <c r="I31" s="5" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="J31" s="3">
         <v>1711</v>
@@ -2049,7 +2043,7 @@
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
       <c r="I32" s="5" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="J32" s="3">
         <v>1711</v>
@@ -2086,7 +2080,7 @@
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
       <c r="I33" s="5" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="J33" s="3">
         <v>1995</v>
@@ -2146,7 +2140,7 @@
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
       <c r="I35" s="5" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="J35" s="3"/>
       <c r="K35" s="3"/>
@@ -2169,10 +2163,10 @@
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
       <c r="I36" s="5" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="K36" s="3"/>
       <c r="L36" s="3"/>
@@ -2194,10 +2188,10 @@
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
       <c r="I37" s="5" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="K37" s="3"/>
       <c r="L37" s="3"/>
@@ -2212,17 +2206,17 @@
         <v>80</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="D38" s="3"/>
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
       <c r="G38" s="3"/>
       <c r="I38" s="5" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="J38" s="3" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="K38" s="3"/>
       <c r="L38" s="3"/>
@@ -2240,10 +2234,10 @@
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
       <c r="I39" s="5" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="J39" s="3" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="K39" s="3"/>
       <c r="L39" s="3"/>
@@ -2304,7 +2298,7 @@
         <v>80</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="D44" s="3"/>
       <c r="E44" s="3"/>
@@ -2328,7 +2322,7 @@
         <v>80</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="D46" s="3"/>
       <c r="E46" s="3"/>
@@ -2787,6 +2781,17 @@
         <v>44</v>
       </c>
     </row>
+    <row r="7" spans="1:41" x14ac:dyDescent="0.35">
+      <c r="I7" s="4"/>
+      <c r="J7" s="4"/>
+      <c r="K7" s="4"/>
+      <c r="L7" s="4"/>
+      <c r="M7" s="4"/>
+      <c r="N7" s="4"/>
+      <c r="O7" s="4"/>
+      <c r="P7" s="4"/>
+      <c r="Q7" s="4"/>
+    </row>
     <row r="8" spans="1:41" x14ac:dyDescent="0.35">
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
@@ -2794,6 +2799,17 @@
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
+      <c r="I8" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
+      <c r="N8" s="3"/>
+      <c r="O8" s="3"/>
+      <c r="P8" s="3"/>
+      <c r="Q8" s="3"/>
     </row>
     <row r="9" spans="1:41" x14ac:dyDescent="0.35">
       <c r="B9" s="5" t="s">
@@ -2806,15 +2822,15 @@
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4"/>
-      <c r="K9" s="4"/>
-      <c r="L9" s="4"/>
-      <c r="M9" s="4"/>
-      <c r="N9" s="4"/>
-      <c r="O9" s="4"/>
-      <c r="P9" s="4"/>
-      <c r="Q9" s="4"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="3"/>
+      <c r="M9" s="3"/>
+      <c r="N9" s="3"/>
+      <c r="O9" s="3"/>
+      <c r="P9" s="3"/>
+      <c r="Q9" s="3"/>
     </row>
     <row r="10" spans="1:41" x14ac:dyDescent="0.35">
       <c r="B10" s="5"/>
@@ -2824,9 +2840,11 @@
       <c r="F10" s="3"/>
       <c r="G10" s="3"/>
       <c r="I10" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="J10" s="3"/>
+        <v>98</v>
+      </c>
+      <c r="J10" s="3">
+        <v>1</v>
+      </c>
       <c r="K10" s="3"/>
       <c r="L10" s="3"/>
       <c r="M10" s="3"/>
@@ -2846,8 +2864,12 @@
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
-      <c r="I11" s="5"/>
-      <c r="J11" s="3"/>
+      <c r="I11" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="J11" s="3">
+        <v>6</v>
+      </c>
       <c r="K11" s="3"/>
       <c r="L11" s="3"/>
       <c r="M11" s="3"/>
@@ -2868,10 +2890,10 @@
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
       <c r="I12" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="J12" s="3">
-        <v>1</v>
+        <v>0.05</v>
       </c>
       <c r="K12" s="3"/>
       <c r="L12" s="3"/>
@@ -2888,12 +2910,8 @@
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
-      <c r="I13" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="J13" s="3">
-        <v>6</v>
-      </c>
+      <c r="I13" s="5"/>
+      <c r="J13" s="3"/>
       <c r="K13" s="3"/>
       <c r="L13" s="3"/>
       <c r="M13" s="3"/>
@@ -2920,15 +2938,23 @@
       </c>
       <c r="G14" s="3"/>
       <c r="I14" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="J14" s="3">
-        <v>0.05</v>
-      </c>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3"/>
-      <c r="M14" s="3"/>
-      <c r="N14" s="3"/>
+        <v>137</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="K14" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="L14" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="M14" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="N14" s="3" t="s">
+        <v>105</v>
+      </c>
       <c r="O14" s="3"/>
       <c r="P14" s="3"/>
       <c r="Q14" s="3"/>
@@ -2978,22 +3004,22 @@
       </c>
       <c r="G16" s="3"/>
       <c r="I16" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="J16" s="3" t="s">
-        <v>102</v>
+        <v>106</v>
+      </c>
+      <c r="J16" s="3">
+        <v>525</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>103</v>
+        <v>174</v>
       </c>
       <c r="L16" s="3" t="s">
-        <v>104</v>
+        <v>59</v>
       </c>
       <c r="M16" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="N16" s="3" t="s">
-        <v>106</v>
+        <v>58</v>
+      </c>
+      <c r="N16" s="3">
+        <v>0.93879999999999997</v>
       </c>
       <c r="O16" s="3"/>
       <c r="P16" s="3"/>
@@ -3016,12 +3042,24 @@
         <v>59</v>
       </c>
       <c r="G17" s="3"/>
-      <c r="I17" s="5"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="3"/>
-      <c r="L17" s="3"/>
-      <c r="M17" s="3"/>
-      <c r="N17" s="3"/>
+      <c r="I17" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="J17" s="3">
+        <v>1050</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="L17" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="M17" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="N17" s="3">
+        <v>0.65800000000000003</v>
+      </c>
       <c r="O17" s="3"/>
       <c r="P17" s="3"/>
       <c r="Q17" s="3"/>
@@ -3034,13 +3072,13 @@
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
       <c r="I18" s="5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="J18" s="3">
-        <v>525</v>
+        <v>-735</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>108</v>
+        <v>176</v>
       </c>
       <c r="L18" s="3" t="s">
         <v>59</v>
@@ -3049,7 +3087,7 @@
         <v>58</v>
       </c>
       <c r="N18" s="3">
-        <v>0.99329999999999996</v>
+        <v>0.85089999999999999</v>
       </c>
       <c r="O18" s="3"/>
       <c r="P18" s="3"/>
@@ -3078,10 +3116,10 @@
         <v>109</v>
       </c>
       <c r="J19" s="3">
-        <v>1050</v>
+        <v>525</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>110</v>
+        <v>174</v>
       </c>
       <c r="L19" s="3" t="s">
         <v>59</v>
@@ -3090,7 +3128,7 @@
         <v>58</v>
       </c>
       <c r="N19" s="3">
-        <v>0.82550000000000001</v>
+        <v>0.93879999999999997</v>
       </c>
       <c r="O19" s="3"/>
       <c r="P19" s="3"/>
@@ -3116,13 +3154,13 @@
         <v>68</v>
       </c>
       <c r="I20" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J20" s="3">
-        <v>-735</v>
+        <v>-1260</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>112</v>
+        <v>177</v>
       </c>
       <c r="L20" s="3" t="s">
         <v>59</v>
@@ -3131,7 +3169,7 @@
         <v>58</v>
       </c>
       <c r="N20" s="3">
-        <v>0.9627</v>
+        <v>0.51339999999999997</v>
       </c>
       <c r="O20" s="3"/>
       <c r="P20" s="3"/>
@@ -3157,13 +3195,13 @@
         <v>70</v>
       </c>
       <c r="I21" s="5" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="J21" s="3">
-        <v>525</v>
+        <v>-1785</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>108</v>
+        <v>178</v>
       </c>
       <c r="L21" s="3" t="s">
         <v>59</v>
@@ -3172,7 +3210,7 @@
         <v>58</v>
       </c>
       <c r="N21" s="3">
-        <v>0.99329999999999996</v>
+        <v>0.2122</v>
       </c>
       <c r="O21" s="3"/>
       <c r="P21" s="3"/>
@@ -3197,24 +3235,12 @@
       <c r="G22" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="I22" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="J22" s="3">
-        <v>-1260</v>
-      </c>
-      <c r="K22" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="L22" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="M22" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="N22" s="3">
-        <v>0.67420000000000002</v>
-      </c>
+      <c r="I22" s="5"/>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
+      <c r="L22" s="3"/>
+      <c r="M22" s="3"/>
+      <c r="N22" s="3"/>
       <c r="O22" s="3"/>
       <c r="P22" s="3"/>
       <c r="Q22" s="3"/>
@@ -3234,24 +3260,12 @@
       </c>
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
-      <c r="I23" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="J23" s="3">
-        <v>-1785</v>
-      </c>
-      <c r="K23" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="L23" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="M23" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="N23" s="3">
-        <v>0.28160000000000002</v>
-      </c>
+      <c r="I23" s="5"/>
+      <c r="J23" s="3"/>
+      <c r="K23" s="3"/>
+      <c r="L23" s="3"/>
+      <c r="M23" s="3"/>
+      <c r="N23" s="3"/>
       <c r="O23" s="3"/>
       <c r="P23" s="3"/>
       <c r="Q23" s="3"/>
@@ -3269,15 +3283,33 @@
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
-      <c r="I24" s="5"/>
-      <c r="J24" s="3"/>
-      <c r="K24" s="3"/>
-      <c r="L24" s="3"/>
-      <c r="M24" s="3"/>
-      <c r="N24" s="3"/>
-      <c r="O24" s="3"/>
-      <c r="P24" s="3"/>
-      <c r="Q24" s="3"/>
+      <c r="I24" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="J24" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="K24" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="L24" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="M24" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="N24" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="O24" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="P24" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="Q24" s="3" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="25" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B25" s="5"/>
@@ -3306,31 +3338,31 @@
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
       <c r="I26" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="J26" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="K26" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="L26" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="M26" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="N26" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="O26" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="P26" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="Q26" s="3" t="s">
-        <v>64</v>
+        <v>106</v>
+      </c>
+      <c r="J26" s="3">
+        <v>8400</v>
+      </c>
+      <c r="K26" s="3">
+        <v>7875</v>
+      </c>
+      <c r="L26" s="3">
+        <v>525</v>
+      </c>
+      <c r="M26" s="3">
+        <v>910.6</v>
+      </c>
+      <c r="N26" s="3">
+        <v>20</v>
+      </c>
+      <c r="O26" s="3">
+        <v>20</v>
+      </c>
+      <c r="P26" s="3">
+        <v>0.81540000000000001</v>
+      </c>
+      <c r="Q26" s="3">
+        <v>76</v>
       </c>
     </row>
     <row r="27" spans="2:17" x14ac:dyDescent="0.35">
@@ -3344,15 +3376,33 @@
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
-      <c r="I27" s="5"/>
-      <c r="J27" s="3"/>
-      <c r="K27" s="3"/>
-      <c r="L27" s="3"/>
-      <c r="M27" s="3"/>
-      <c r="N27" s="3"/>
-      <c r="O27" s="3"/>
-      <c r="P27" s="3"/>
-      <c r="Q27" s="3"/>
+      <c r="I27" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="J27" s="3">
+        <v>8400</v>
+      </c>
+      <c r="K27" s="3">
+        <v>7350</v>
+      </c>
+      <c r="L27" s="3">
+        <v>1050</v>
+      </c>
+      <c r="M27" s="3">
+        <v>910.6</v>
+      </c>
+      <c r="N27" s="3">
+        <v>20</v>
+      </c>
+      <c r="O27" s="3">
+        <v>20</v>
+      </c>
+      <c r="P27" s="3">
+        <v>1.631</v>
+      </c>
+      <c r="Q27" s="3">
+        <v>76</v>
+      </c>
     </row>
     <row r="28" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B28" s="5" t="s">
@@ -3366,16 +3416,16 @@
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
       <c r="I28" s="5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="J28" s="3">
         <v>8400</v>
       </c>
       <c r="K28" s="3">
-        <v>7875</v>
+        <v>9135</v>
       </c>
       <c r="L28" s="3">
-        <v>525</v>
+        <v>-735</v>
       </c>
       <c r="M28" s="3">
         <v>910.6</v>
@@ -3387,7 +3437,7 @@
         <v>20</v>
       </c>
       <c r="P28" s="3">
-        <v>0.57650000000000001</v>
+        <v>1.1419999999999999</v>
       </c>
       <c r="Q28" s="3">
         <v>76</v>
@@ -3408,13 +3458,13 @@
         <v>109</v>
       </c>
       <c r="J29" s="3">
-        <v>8400</v>
+        <v>7875</v>
       </c>
       <c r="K29" s="3">
         <v>7350</v>
       </c>
       <c r="L29" s="3">
-        <v>1050</v>
+        <v>525</v>
       </c>
       <c r="M29" s="3">
         <v>910.6</v>
@@ -3426,7 +3476,7 @@
         <v>20</v>
       </c>
       <c r="P29" s="3">
-        <v>1.153</v>
+        <v>0.81540000000000001</v>
       </c>
       <c r="Q29" s="3">
         <v>76</v>
@@ -3444,16 +3494,16 @@
       <c r="F30" s="3"/>
       <c r="G30" s="3"/>
       <c r="I30" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J30" s="3">
-        <v>8400</v>
+        <v>7875</v>
       </c>
       <c r="K30" s="3">
         <v>9135</v>
       </c>
       <c r="L30" s="3">
-        <v>-735</v>
+        <v>-1260</v>
       </c>
       <c r="M30" s="3">
         <v>910.6</v>
@@ -3465,7 +3515,7 @@
         <v>20</v>
       </c>
       <c r="P30" s="3">
-        <v>0.80720000000000003</v>
+        <v>1.9570000000000001</v>
       </c>
       <c r="Q30" s="3">
         <v>76</v>
@@ -3483,16 +3533,16 @@
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
       <c r="I31" s="5" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="J31" s="3">
-        <v>7875</v>
+        <v>7350</v>
       </c>
       <c r="K31" s="3">
-        <v>7350</v>
+        <v>9135</v>
       </c>
       <c r="L31" s="3">
-        <v>525</v>
+        <v>-1785</v>
       </c>
       <c r="M31" s="3">
         <v>910.6</v>
@@ -3504,7 +3554,7 @@
         <v>20</v>
       </c>
       <c r="P31" s="3">
-        <v>0.57650000000000001</v>
+        <v>2.7719999999999998</v>
       </c>
       <c r="Q31" s="3">
         <v>76</v>
@@ -3517,33 +3567,15 @@
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
-      <c r="I32" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="J32" s="3">
-        <v>7875</v>
-      </c>
-      <c r="K32" s="3">
-        <v>9135</v>
-      </c>
-      <c r="L32" s="3">
-        <v>-1260</v>
-      </c>
-      <c r="M32" s="3">
-        <v>910.6</v>
-      </c>
-      <c r="N32" s="3">
-        <v>20</v>
-      </c>
-      <c r="O32" s="3">
-        <v>20</v>
-      </c>
-      <c r="P32" s="3">
-        <v>1.3839999999999999</v>
-      </c>
-      <c r="Q32" s="3">
-        <v>76</v>
-      </c>
+      <c r="I32" s="5"/>
+      <c r="J32" s="3"/>
+      <c r="K32" s="3"/>
+      <c r="L32" s="3"/>
+      <c r="M32" s="3"/>
+      <c r="N32" s="3"/>
+      <c r="O32" s="3"/>
+      <c r="P32" s="3"/>
+      <c r="Q32" s="3"/>
     </row>
     <row r="33" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B33" s="5" t="s">
@@ -3555,32 +3587,16 @@
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
       <c r="I33" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="J33" s="3">
-        <v>7350</v>
-      </c>
-      <c r="K33" s="3">
-        <v>9135</v>
-      </c>
-      <c r="L33" s="3">
-        <v>-1785</v>
-      </c>
-      <c r="M33" s="3">
-        <v>910.6</v>
-      </c>
-      <c r="N33" s="3">
-        <v>20</v>
-      </c>
-      <c r="O33" s="3">
-        <v>20</v>
-      </c>
-      <c r="P33" s="3">
-        <v>1.96</v>
-      </c>
-      <c r="Q33" s="3">
-        <v>76</v>
-      </c>
+        <v>118</v>
+      </c>
+      <c r="J33" s="3"/>
+      <c r="K33" s="3"/>
+      <c r="L33" s="3"/>
+      <c r="M33" s="3"/>
+      <c r="N33" s="3"/>
+      <c r="O33" s="3"/>
+      <c r="P33" s="3"/>
+      <c r="Q33" s="3"/>
     </row>
     <row r="34" spans="2:17" x14ac:dyDescent="0.35">
       <c r="B34" s="5" t="s">
@@ -3593,8 +3609,12 @@
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
       <c r="G34" s="3"/>
-      <c r="I34" s="5"/>
-      <c r="J34" s="3"/>
+      <c r="I34" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="J34" s="3" t="s">
+        <v>120</v>
+      </c>
       <c r="K34" s="3"/>
       <c r="L34" s="3"/>
       <c r="M34" s="3"/>
@@ -3615,9 +3635,11 @@
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
       <c r="I35" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="J35" s="3"/>
+        <v>121</v>
+      </c>
+      <c r="J35" s="3" t="s">
+        <v>120</v>
+      </c>
       <c r="K35" s="3"/>
       <c r="L35" s="3"/>
       <c r="M35" s="3"/>
@@ -3638,10 +3660,10 @@
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
       <c r="I36" s="5" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="K36" s="3"/>
       <c r="L36" s="3"/>
@@ -3663,10 +3685,10 @@
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
       <c r="I37" s="5" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="K37" s="3"/>
       <c r="L37" s="3"/>
@@ -3687,12 +3709,8 @@
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
       <c r="G38" s="3"/>
-      <c r="I38" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="J38" s="3" t="s">
-        <v>127</v>
-      </c>
+      <c r="I38" s="5"/>
+      <c r="J38" s="3"/>
       <c r="K38" s="3"/>
       <c r="L38" s="3"/>
       <c r="M38" s="3"/>
@@ -3708,12 +3726,8 @@
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
-      <c r="I39" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="J39" s="3" t="s">
-        <v>127</v>
-      </c>
+      <c r="I39" s="5"/>
+      <c r="J39" s="3"/>
       <c r="K39" s="3"/>
       <c r="L39" s="3"/>
       <c r="M39" s="3"/>
@@ -4429,22 +4443,22 @@
       </c>
       <c r="G16" s="3"/>
       <c r="J16" s="5" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="K16" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="L16" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="L16" s="3" t="s">
+      <c r="M16" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="M16" s="3" t="s">
+      <c r="N16" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="N16" s="3" t="s">
+      <c r="O16" s="3" t="s">
         <v>105</v>
-      </c>
-      <c r="O16" s="3" t="s">
-        <v>106</v>
       </c>
       <c r="P16" s="3"/>
       <c r="Q16" s="3"/>
@@ -4485,32 +4499,32 @@
         <v>33.15</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="G18" s="3"/>
       <c r="J18" s="5" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="K18" s="3">
         <v>945</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="N18" s="3" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="O18" s="3" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="P18" s="3"/>
       <c r="Q18" s="3"/>
@@ -4524,13 +4538,13 @@
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
       <c r="J19" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="K19" s="3">
         <v>-105</v>
       </c>
       <c r="L19" s="3" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="M19" s="3" t="s">
         <v>59</v>
@@ -4565,19 +4579,19 @@
         <v>54</v>
       </c>
       <c r="J20" s="5" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="K20" s="3">
         <v>735</v>
       </c>
       <c r="L20" s="3" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="N20" s="3" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="O20" s="3">
         <v>3.0000000000000001E-3</v>
@@ -4600,28 +4614,28 @@
         <v>55125</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="K21" s="3">
         <v>-1050</v>
       </c>
       <c r="L21" s="3" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="M21" s="3" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="N21" s="3" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="O21" s="3" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="P21" s="3"/>
       <c r="Q21" s="3"/>
@@ -4641,19 +4655,19 @@
         <v>496125</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="J22" s="5" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="K22" s="3">
         <v>-210</v>
       </c>
       <c r="L22" s="3" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="M22" s="3" t="s">
         <v>59</v>
@@ -4682,25 +4696,25 @@
         <v>15931125</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="J23" s="5" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="K23" s="3">
         <v>840</v>
       </c>
       <c r="L23" s="3" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="N23" s="3" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="O23" s="3">
         <v>5.0000000000000001E-4</v>
@@ -4765,28 +4779,28 @@
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
       <c r="J26" s="5" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="L26" s="3" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="M26" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="N26" s="3" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="O26" s="3" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="P26" s="3" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="Q26" s="3" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="R26" s="3" t="s">
         <v>64</v>
@@ -4823,7 +4837,7 @@
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
       <c r="J28" s="5" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="K28" s="3">
         <v>2205</v>
@@ -4852,7 +4866,7 @@
     </row>
     <row r="29" spans="2:18" x14ac:dyDescent="0.35">
       <c r="B29" s="5" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="C29" s="3">
         <v>1365</v>
@@ -4862,7 +4876,7 @@
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
       <c r="J29" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="K29" s="3">
         <v>2205</v>
@@ -4901,7 +4915,7 @@
       <c r="F30" s="3"/>
       <c r="G30" s="3"/>
       <c r="J30" s="5" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="K30" s="3">
         <v>2205</v>
@@ -4940,7 +4954,7 @@
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
       <c r="J31" s="5" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="K31" s="3">
         <v>1260</v>
@@ -4972,14 +4986,14 @@
         <v>80</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="D32" s="3"/>
       <c r="E32" s="3"/>
       <c r="F32" s="3"/>
       <c r="G32" s="3"/>
       <c r="J32" s="5" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="K32" s="3">
         <v>1260</v>
@@ -5014,7 +5028,7 @@
       <c r="F33" s="3"/>
       <c r="G33" s="3"/>
       <c r="J33" s="5" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="K33" s="3">
         <v>2310</v>
@@ -5072,7 +5086,7 @@
       <c r="F35" s="3"/>
       <c r="G35" s="3"/>
       <c r="J35" s="5" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="K35" s="3"/>
       <c r="L35" s="3"/>
@@ -5095,10 +5109,10 @@
       <c r="F36" s="3"/>
       <c r="G36" s="3"/>
       <c r="J36" s="5" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="K36" s="3" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="L36" s="3"/>
       <c r="M36" s="3"/>
@@ -5120,10 +5134,10 @@
       <c r="F37" s="3"/>
       <c r="G37" s="3"/>
       <c r="J37" s="5" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="K37" s="3" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="L37" s="3"/>
       <c r="M37" s="3"/>
@@ -5145,10 +5159,10 @@
       <c r="F38" s="3"/>
       <c r="G38" s="3"/>
       <c r="J38" s="5" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="K38" s="3" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="L38" s="3"/>
       <c r="M38" s="3"/>
@@ -5163,17 +5177,17 @@
         <v>80</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="D39" s="3"/>
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
       <c r="G39" s="3"/>
       <c r="J39" s="5" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="K39" s="3" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="L39" s="3"/>
       <c r="M39" s="3"/>
@@ -5242,7 +5256,7 @@
         <v>80</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="D45" s="3"/>
       <c r="E45" s="3"/>
@@ -5266,7 +5280,7 @@
         <v>80</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="D47" s="3"/>
       <c r="E47" s="3"/>

</xml_diff>